<commit_message>
Update formulas to modern Excel syntax (LET, FILTER, SORT)
- Replace nested IF/INDEX/MATCH with LET for named variables
- Use FILTER for dynamic array filtering instead of SUMPRODUCT
- Use SORT for automatic sorting of results
- Use HSTACK for combining arrays
- Interest calculations use LET for clarity
- All formulas optimized for Excel 365/2021+

Modern formula features:
- LET() defines named variables within formulas
- FILTER() returns arrays meeting criteria
- SORT() sorts arrays by column
- HSTACK() horizontally stacks arrays
</commit_message>
<xml_diff>
--- a/Cash_Management_Controller.xlsx
+++ b/Cash_Management_Controller.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -184,6 +184,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00007AFF"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -561,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -689,11 +695,12 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -723,14 +730,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="00E3F2FD"/>
           <bgColor rgb="00E3F2FD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F5F5F7"/>
-          <bgColor rgb="00F5F5F7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1166,12 +1165,12 @@
       </c>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="8">
-        <f>SUMIF(PaymentsData!F:F,"Pending",PaymentsData!D:D)</f>
+        <f>LET(status,PaymentsData!F:F,amounts,PaymentsData!D:D,SUMIF(status,"Pending",amounts))</f>
         <v/>
       </c>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="9">
-        <f>SUMIF(DepositsData!G:G,"Active",DepositsData!D:D)</f>
+        <f>LET(status,DepositsData!G:G,principal,DepositsData!D:D,SUMIF(status,"Active",principal))</f>
         <v/>
       </c>
       <c r="G6" s="7" t="n"/>
@@ -1197,12 +1196,12 @@
       </c>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="14">
-        <f>COUNTIF(PaymentsData!F:F,"Pending")&amp;" payments"</f>
+        <f>LET(status,PaymentsData!F:F,COUNTIF(status,"Pending")&amp;" payments")</f>
         <v/>
       </c>
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="14">
-        <f>COUNTIF(DepositsData!G:G,"Active")&amp;" deposits"</f>
+        <f>LET(status,DepositsData!G:G,COUNTIF(status,"Active")&amp;" deposits")</f>
         <v/>
       </c>
       <c r="G8" s="15" t="n"/>
@@ -1263,151 +1262,446 @@
     </row>
     <row r="12">
       <c r="B12" s="20">
-        <f>IFERROR(INDEX(PaymentsData!B:B,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),1)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,1,1),"")
+)</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),1)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,1,2),"")
+)</f>
         <v/>
       </c>
       <c r="D12" s="22">
-        <f>IFERROR(INDEX(PaymentsData!D:D,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),1)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,1,3),"")
+)</f>
         <v/>
       </c>
       <c r="E12" s="21">
-        <f>IFERROR(INDEX(PaymentsData!E:E,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),1)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,1,4),"")
+)</f>
         <v/>
       </c>
       <c r="F12" s="21">
-        <f>IFERROR(INDEX(PaymentsData!F:F,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),1)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,1,5),"")
+)</f>
         <v/>
       </c>
       <c r="G12" s="20">
-        <f>IFERROR(INDEX(DepositsData!F:F,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),1)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,1,1),"")
+)</f>
         <v/>
       </c>
       <c r="H12" s="23">
-        <f>IFERROR(INDEX(DepositsData!D:D,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),1)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,1,2),"")
+)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="20">
-        <f>IFERROR(INDEX(PaymentsData!B:B,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),2)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,2,1),"")
+)</f>
         <v/>
       </c>
       <c r="C13" s="21">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),2)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,2,2),"")
+)</f>
         <v/>
       </c>
       <c r="D13" s="22">
-        <f>IFERROR(INDEX(PaymentsData!D:D,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),2)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,2,3),"")
+)</f>
         <v/>
       </c>
       <c r="E13" s="21">
-        <f>IFERROR(INDEX(PaymentsData!E:E,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),2)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,2,4),"")
+)</f>
         <v/>
       </c>
       <c r="F13" s="21">
-        <f>IFERROR(INDEX(PaymentsData!F:F,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),2)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,2,5),"")
+)</f>
         <v/>
       </c>
       <c r="G13" s="20">
-        <f>IFERROR(INDEX(DepositsData!F:F,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),2)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,2,1),"")
+)</f>
         <v/>
       </c>
       <c r="H13" s="23">
-        <f>IFERROR(INDEX(DepositsData!D:D,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),2)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,2,2),"")
+)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="20">
-        <f>IFERROR(INDEX(PaymentsData!B:B,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),3)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,3,1),"")
+)</f>
         <v/>
       </c>
       <c r="C14" s="21">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),3)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,3,2),"")
+)</f>
         <v/>
       </c>
       <c r="D14" s="22">
-        <f>IFERROR(INDEX(PaymentsData!D:D,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),3)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,3,3),"")
+)</f>
         <v/>
       </c>
       <c r="E14" s="21">
-        <f>IFERROR(INDEX(PaymentsData!E:E,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),3)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,3,4),"")
+)</f>
         <v/>
       </c>
       <c r="F14" s="21">
-        <f>IFERROR(INDEX(PaymentsData!F:F,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),3)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,3,5),"")
+)</f>
         <v/>
       </c>
       <c r="G14" s="20">
-        <f>IFERROR(INDEX(DepositsData!F:F,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),3)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,3,1),"")
+)</f>
         <v/>
       </c>
       <c r="H14" s="23">
-        <f>IFERROR(INDEX(DepositsData!D:D,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),3)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,3,2),"")
+)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="20">
-        <f>IFERROR(INDEX(PaymentsData!B:B,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),4)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,4,1),"")
+)</f>
         <v/>
       </c>
       <c r="C15" s="21">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),4)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,4,2),"")
+)</f>
         <v/>
       </c>
       <c r="D15" s="22">
-        <f>IFERROR(INDEX(PaymentsData!D:D,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),4)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,4,3),"")
+)</f>
         <v/>
       </c>
       <c r="E15" s="21">
-        <f>IFERROR(INDEX(PaymentsData!E:E,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),4)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,4,4),"")
+)</f>
         <v/>
       </c>
       <c r="F15" s="21">
-        <f>IFERROR(INDEX(PaymentsData!F:F,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),4)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,4,5),"")
+)</f>
         <v/>
       </c>
       <c r="G15" s="20">
-        <f>IFERROR(INDEX(DepositsData!F:F,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),4)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,4,1),"")
+)</f>
         <v/>
       </c>
       <c r="H15" s="23">
-        <f>IFERROR(INDEX(DepositsData!D:D,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),4)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,4,2),"")
+)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="20">
-        <f>IFERROR(INDEX(PaymentsData!B:B,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),5)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,5,1),"")
+)</f>
         <v/>
       </c>
       <c r="C16" s="21">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),5)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,5,2),"")
+)</f>
         <v/>
       </c>
       <c r="D16" s="22">
-        <f>IFERROR(INDEX(PaymentsData!D:D,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),5)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,5,3),"")
+)</f>
         <v/>
       </c>
       <c r="E16" s="21">
-        <f>IFERROR(INDEX(PaymentsData!E:E,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),5)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,5,4),"")
+)</f>
         <v/>
       </c>
       <c r="F16" s="21">
-        <f>IFERROR(INDEX(PaymentsData!F:F,SMALL(IF((PaymentsData!B:B&gt;=TODAY())*(PaymentsData!B:B&lt;=TODAY()+7),ROW(PaymentsData!B:B)),5)),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    categories,PaymentsData!E2:E500,
+    statuses,PaymentsData!F2:F500,
+    upcoming,FILTER(HSTACK(dates,payees,amounts,categories,statuses),(dates&gt;=TODAY())*(dates&lt;=TODAY()+7),""),
+    sorted,SORT(upcoming,1,1),
+    IFERROR(INDEX(sorted,5,5),"")
+)</f>
         <v/>
       </c>
       <c r="G16" s="20">
-        <f>IFERROR(INDEX(DepositsData!F:F,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),5)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,5,1),"")
+)</f>
         <v/>
       </c>
       <c r="H16" s="23">
-        <f>IFERROR(INDEX(DepositsData!D:D,SMALL(IF((DepositsData!F:F&gt;=TODAY())*(DepositsData!F:F&lt;=TODAY()+30)*(DepositsData!G:G="Active"),ROW(DepositsData!F:F)),5)),"")</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    maturing,FILTER(HSTACK(maturity,principal),(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),""),
+    sorted,SORT(maturing,1,1),
+    IFERROR(INDEX(sorted,5,2),"")
+)</f>
         <v/>
       </c>
     </row>
@@ -1616,6 +1910,7 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="3" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1"/>
@@ -1706,27 +2001,63 @@
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="32" t="n"/>
       <c r="C8" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=1,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=1,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=1,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D8" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=2,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=2,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=2,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E8" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=3,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=3,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=3,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F8" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=4,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=4,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=4,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G8" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=5,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=5,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=5,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H8" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=6,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=6,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=6,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="J8" s="34" t="inlineStr">
@@ -1743,27 +2074,63 @@
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="32" t="n"/>
       <c r="C9" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=1,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=1,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=1,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D9" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=2,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=2,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=2,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E9" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=3,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=3,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=3,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F9" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=4,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=4,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=4,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G9" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=5,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=5,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=5,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H9" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=6,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=6,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=6,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="J9" s="36" t="inlineStr">
@@ -1780,27 +2147,63 @@
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="32" t="n"/>
       <c r="C10" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=1,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=1,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=1,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D10" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=2,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=2,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=2,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E10" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=3,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=3,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=3,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F10" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=4,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=4,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=4,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G10" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=5,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=5,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=5,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H10" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=6,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=6,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=6,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="J10" s="37" t="inlineStr">
@@ -1868,91 +2271,217 @@
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=7,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=7,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=7,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C13" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=8,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=8,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=8,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D13" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=9,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=9,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=9,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E13" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=10,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=10,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=10,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F13" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=11,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=11,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=11,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G13" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=12,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=12,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=12,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H13" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=13,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=13,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=13,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="B14" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=7,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=7,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=7,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C14" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=8,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=8,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=8,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D14" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=9,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=9,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=9,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E14" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=10,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=10,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=10,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F14" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=11,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=11,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=11,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G14" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=12,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=12,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=12,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H14" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=13,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=13,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=13,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="B15" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=7,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=7,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=7,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C15" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=8,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=8,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=8,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D15" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=9,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=9,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=9,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E15" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=10,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=10,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=10,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F15" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=11,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=11,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=11,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G15" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=12,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=12,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=12,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H15" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=13,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=13,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=13,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="J15" s="17" t="inlineStr">
@@ -1975,7 +2504,7 @@
         </is>
       </c>
       <c r="K16" s="43">
-        <f>SUMIF(PaymentsData!F:F,"Scheduled",PaymentsData!D:D)</f>
+        <f>LET(s,PaymentsData!F:F,a,PaymentsData!D:D,SUMIF(s,"Scheduled",a))</f>
         <v/>
       </c>
     </row>
@@ -2007,37 +2536,79 @@
         </is>
       </c>
       <c r="K17" s="43">
-        <f>SUMIF(PaymentsData!F:F,"Pending",PaymentsData!D:D)</f>
+        <f>LET(s,PaymentsData!F:F,a,PaymentsData!D:D,SUMIF(s,"Pending",a))</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=14,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=14,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=14,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C18" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=15,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=15,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=15,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D18" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=16,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=16,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=16,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E18" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=17,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=17,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=17,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F18" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=18,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=18,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=18,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G18" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=19,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=19,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=19,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H18" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=20,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=20,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=20,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="J18" s="35" t="inlineStr">
@@ -2046,37 +2617,79 @@
         </is>
       </c>
       <c r="K18" s="43">
-        <f>SUMIF(PaymentsData!F:F,"Paid",PaymentsData!D:D)</f>
+        <f>LET(s,PaymentsData!F:F,a,PaymentsData!D:D,SUMIF(s,"Paid",a))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=14,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=14,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=14,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C19" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=15,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=15,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=15,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D19" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=16,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=16,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=16,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E19" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=17,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=17,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=17,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F19" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=18,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=18,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=18,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G19" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=19,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=19,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=19,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H19" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=20,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=20,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=20,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="J19" s="35" t="inlineStr">
@@ -2085,37 +2698,79 @@
         </is>
       </c>
       <c r="K19" s="44">
-        <f>SUMIF(PaymentsData!F:F,"Overdue",PaymentsData!D:D)</f>
+        <f>LET(s,PaymentsData!F:F,a,PaymentsData!D:D,SUMIF(s,"Overdue",a))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=14,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=14,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=14,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C20" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=15,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=15,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=15,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D20" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=16,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=16,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=16,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E20" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=17,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=17,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=17,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F20" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=18,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=18,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=18,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G20" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=19,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=19,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=19,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H20" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=20,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=20,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=20,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
     </row>
@@ -2153,91 +2808,217 @@
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=21,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=21,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=21,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C23" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=22,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=22,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=22,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D23" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=23,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=23,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=23,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E23" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=24,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=24,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=24,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F23" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=25,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=25,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=25,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G23" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=26,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=26,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=26,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H23" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=27,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=27,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=27,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=21,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=21,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=21,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C24" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=22,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=22,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=22,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D24" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=23,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=23,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=23,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E24" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=24,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=24,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=24,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F24" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=25,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=25,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=25,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G24" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=26,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=26,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=26,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H24" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=27,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=27,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=27,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=21,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=21,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=21,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C25" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=22,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=22,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=22,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D25" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=23,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=23,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=23,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E25" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=24,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=24,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=24,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F25" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=25,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=25,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=25,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="G25" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=26,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=26,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=26,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="H25" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=27,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=27,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=27,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
     </row>
@@ -2269,19 +3050,43 @@
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=28,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=28,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=28,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C28" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=29,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=29,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=29,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D28" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=30,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=30,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=30,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E28" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=31,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=31,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),1)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=31,""),
+    IFERROR(INDEX(dayPayments,1,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,1,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F28" s="32" t="n"/>
@@ -2290,19 +3095,43 @@
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=28,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=28,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=28,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C29" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=29,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=29,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=29,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D29" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=30,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=30,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=30,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E29" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=31,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=31,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),2)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=31,""),
+    IFERROR(INDEX(dayPayments,2,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,2,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F29" s="32" t="n"/>
@@ -2311,19 +3140,43 @@
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=28,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=28,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=28,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="C30" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=29,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=29,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=29,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="D30" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=30,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=30,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=30,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="E30" s="33">
-        <f>IFERROR(INDEX(PaymentsData!C:C,SMALL(IF(DAY(PaymentsData!B:B)=31,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3))&amp;" - $"&amp;TEXT(INDEX(PaymentsData!D:D,SMALL(IF(DAY(PaymentsData!B:B)=31,IF(MONTH(PaymentsData!B:B)=MONTH(C4),ROW(PaymentsData!B:B))),3)),"#,##0"),"")</f>
+        <f>LET(
+    dates,PaymentsData!B2:B500,
+    payees,PaymentsData!C2:C500,
+    amounts,PaymentsData!D2:D500,
+    dayPayments,FILTER(HSTACK(payees,amounts),DAY(dates)=31,""),
+    IFERROR(INDEX(dayPayments,3,1)&amp;" $"&amp;TEXT(INDEX(dayPayments,3,2),"#,##0"),"")
+)</f>
         <v/>
       </c>
       <c r="F30" s="32" t="n"/>
@@ -2430,22 +3283,28 @@
     </row>
     <row r="6">
       <c r="B6" s="46">
-        <f>SUMIF(DepositsData!G:G,"Active",DepositsData!D:D)</f>
+        <f>LET(status,DepositsData!G:G,principal,DepositsData!D:D,SUMIF(status,"Active",principal))</f>
         <v/>
       </c>
       <c r="C6" s="47" t="n"/>
       <c r="D6" s="48">
-        <f>AVERAGEIF(DepositsData!G:G,"Active",DepositsData!E:E)</f>
+        <f>LET(status,DepositsData!G:G,rates,DepositsData!E:E,AVERAGEIF(status,"Active",rates))</f>
         <v/>
       </c>
       <c r="E6" s="47" t="n"/>
       <c r="F6" s="49">
-        <f>SUMIF(DepositsData!G:G,"Active",DepositsData!H:H)</f>
+        <f>LET(status,DepositsData!G:G,interest,DepositsData!H:H,SUMIF(status,"Active",interest))</f>
         <v/>
       </c>
       <c r="G6" s="47" t="n"/>
       <c r="H6" s="50">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;=TODAY())*(DepositsData!F2:F100&lt;=TODAY()+30)*(DepositsData!G2:G100="Active")*DepositsData!D2:D100)</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    filtered,FILTER(principal,(maturity&gt;=TODAY())*(maturity&lt;=TODAY()+30)*(status="Active"),0),
+    SUM(filtered)
+)</f>
         <v/>
       </c>
       <c r="I6" s="47" t="n"/>
@@ -2540,7 +3399,7 @@
         <v/>
       </c>
       <c r="H11" s="53">
-        <f>IF(DepositsData!F2="","",MAX(0,DepositsData!F2-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F2,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I11" s="54">
@@ -2578,7 +3437,7 @@
         <v/>
       </c>
       <c r="H12" s="53">
-        <f>IF(DepositsData!F3="","",MAX(0,DepositsData!F3-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F3,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I12" s="54">
@@ -2616,7 +3475,7 @@
         <v/>
       </c>
       <c r="H13" s="53">
-        <f>IF(DepositsData!F4="","",MAX(0,DepositsData!F4-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F4,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I13" s="54">
@@ -2654,7 +3513,7 @@
         <v/>
       </c>
       <c r="H14" s="53">
-        <f>IF(DepositsData!F5="","",MAX(0,DepositsData!F5-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F5,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I14" s="54">
@@ -2692,7 +3551,7 @@
         <v/>
       </c>
       <c r="H15" s="53">
-        <f>IF(DepositsData!F6="","",MAX(0,DepositsData!F6-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F6,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I15" s="54">
@@ -2730,7 +3589,7 @@
         <v/>
       </c>
       <c r="H16" s="53">
-        <f>IF(DepositsData!F7="","",MAX(0,DepositsData!F7-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F7,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I16" s="54">
@@ -2768,7 +3627,7 @@
         <v/>
       </c>
       <c r="H17" s="53">
-        <f>IF(DepositsData!F8="","",MAX(0,DepositsData!F8-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F8,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I17" s="54">
@@ -2806,7 +3665,7 @@
         <v/>
       </c>
       <c r="H18" s="53">
-        <f>IF(DepositsData!F9="","",MAX(0,DepositsData!F9-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F9,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I18" s="54">
@@ -2844,7 +3703,7 @@
         <v/>
       </c>
       <c r="H19" s="53">
-        <f>IF(DepositsData!F10="","",MAX(0,DepositsData!F10-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F10,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I19" s="54">
@@ -2882,7 +3741,7 @@
         <v/>
       </c>
       <c r="H20" s="53">
-        <f>IF(DepositsData!F11="","",MAX(0,DepositsData!F11-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F11,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I20" s="54">
@@ -2920,7 +3779,7 @@
         <v/>
       </c>
       <c r="H21" s="53">
-        <f>IF(DepositsData!F12="","",MAX(0,DepositsData!F12-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F12,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I21" s="54">
@@ -2958,7 +3817,7 @@
         <v/>
       </c>
       <c r="H22" s="53">
-        <f>IF(DepositsData!F13="","",MAX(0,DepositsData!F13-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F13,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I22" s="54">
@@ -2996,7 +3855,7 @@
         <v/>
       </c>
       <c r="H23" s="53">
-        <f>IF(DepositsData!F14="","",MAX(0,DepositsData!F14-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F14,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I23" s="54">
@@ -3034,7 +3893,7 @@
         <v/>
       </c>
       <c r="H24" s="53">
-        <f>IF(DepositsData!F15="","",MAX(0,DepositsData!F15-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F15,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I24" s="54">
@@ -3072,7 +3931,7 @@
         <v/>
       </c>
       <c r="H25" s="53">
-        <f>IF(DepositsData!F16="","",MAX(0,DepositsData!F16-TODAY()))</f>
+        <f>LET(maturity,DepositsData!F16,IF(maturity="","",MAX(0,maturity-TODAY())))</f>
         <v/>
       </c>
       <c r="I25" s="54">
@@ -3120,15 +3979,27 @@
         </is>
       </c>
       <c r="C30" s="58">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;=TODAY())*(DepositsData!F2:F100&lt;=TODAY()+30)*(DepositsData!G2:G100="Active"))</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    ROWS(FILTER(maturity,(daysToMaturity&gt;=0)*(daysToMaturity&lt;=30)*(status="Active"),{}))
+)</f>
         <v/>
       </c>
       <c r="D30" s="25">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;=TODAY())*(DepositsData!F2:F100&lt;=TODAY()+30)*(DepositsData!G2:G100="Active")*DepositsData!D2:D100)</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    filtered,FILTER(principal,(daysToMaturity&gt;=0)*(daysToMaturity&lt;=30)*(status="Active"),0),
+    SUM(filtered)
+)</f>
         <v/>
       </c>
       <c r="E30" s="59">
-        <f>IFERROR(D30/SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),0)</f>
+        <f>LET(amt,D30,total,SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),IFERROR(amt/total,0))</f>
         <v/>
       </c>
     </row>
@@ -3139,15 +4010,27 @@
         </is>
       </c>
       <c r="C31" s="58">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;TODAY()+30)*(DepositsData!F2:F100&lt;=TODAY()+60)*(DepositsData!G2:G100="Active"))</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    ROWS(FILTER(maturity,(daysToMaturity&gt;=31)*(daysToMaturity&lt;=60)*(status="Active"),{}))
+)</f>
         <v/>
       </c>
       <c r="D31" s="25">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;TODAY()+30)*(DepositsData!F2:F100&lt;=TODAY()+60)*(DepositsData!G2:G100="Active")*DepositsData!D2:D100)</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    filtered,FILTER(principal,(daysToMaturity&gt;=31)*(daysToMaturity&lt;=60)*(status="Active"),0),
+    SUM(filtered)
+)</f>
         <v/>
       </c>
       <c r="E31" s="59">
-        <f>IFERROR(D31/SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),0)</f>
+        <f>LET(amt,D31,total,SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),IFERROR(amt/total,0))</f>
         <v/>
       </c>
     </row>
@@ -3158,15 +4041,27 @@
         </is>
       </c>
       <c r="C32" s="58">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;TODAY()+60)*(DepositsData!F2:F100&lt;=TODAY()+90)*(DepositsData!G2:G100="Active"))</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    ROWS(FILTER(maturity,(daysToMaturity&gt;=61)*(daysToMaturity&lt;=90)*(status="Active"),{}))
+)</f>
         <v/>
       </c>
       <c r="D32" s="25">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;TODAY()+60)*(DepositsData!F2:F100&lt;=TODAY()+90)*(DepositsData!G2:G100="Active")*DepositsData!D2:D100)</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    filtered,FILTER(principal,(daysToMaturity&gt;=61)*(daysToMaturity&lt;=90)*(status="Active"),0),
+    SUM(filtered)
+)</f>
         <v/>
       </c>
       <c r="E32" s="59">
-        <f>IFERROR(D32/SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),0)</f>
+        <f>LET(amt,D32,total,SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),IFERROR(amt/total,0))</f>
         <v/>
       </c>
     </row>
@@ -3177,15 +4072,27 @@
         </is>
       </c>
       <c r="C33" s="58">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;TODAY()+90)*(DepositsData!F2:F100&lt;=TODAY()+180)*(DepositsData!G2:G100="Active"))</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    ROWS(FILTER(maturity,(daysToMaturity&gt;=91)*(daysToMaturity&lt;=180)*(status="Active"),{}))
+)</f>
         <v/>
       </c>
       <c r="D33" s="25">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;TODAY()+90)*(DepositsData!F2:F100&lt;=TODAY()+180)*(DepositsData!G2:G100="Active")*DepositsData!D2:D100)</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    filtered,FILTER(principal,(daysToMaturity&gt;=91)*(daysToMaturity&lt;=180)*(status="Active"),0),
+    SUM(filtered)
+)</f>
         <v/>
       </c>
       <c r="E33" s="59">
-        <f>IFERROR(D33/SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),0)</f>
+        <f>LET(amt,D33,total,SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),IFERROR(amt/total,0))</f>
         <v/>
       </c>
     </row>
@@ -3196,15 +4103,27 @@
         </is>
       </c>
       <c r="C34" s="58">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;TODAY()+180)*(DepositsData!G2:G100="Active"))</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    ROWS(FILTER(maturity,(daysToMaturity&gt;=181)*(daysToMaturity&lt;=9999)*(status="Active"),{}))
+)</f>
         <v/>
       </c>
       <c r="D34" s="25">
-        <f>SUMPRODUCT((DepositsData!F2:F100&gt;TODAY()+180)*(DepositsData!G2:G100="Active")*DepositsData!D2:D100)</f>
+        <f>LET(
+    maturity,DepositsData!F2:F100,
+    principal,DepositsData!D2:D100,
+    status,DepositsData!G2:G100,
+    daysToMaturity,maturity-TODAY(),
+    filtered,FILTER(principal,(daysToMaturity&gt;=181)*(daysToMaturity&lt;=9999)*(status="Active"),0),
+    SUM(filtered)
+)</f>
         <v/>
       </c>
       <c r="E34" s="59">
-        <f>IFERROR(D34/SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),0)</f>
+        <f>LET(amt,D34,total,SUMIF(DepositsData!G:G,"Active",DepositsData!D:D),IFERROR(amt/total,0))</f>
         <v/>
       </c>
     </row>
@@ -3326,11 +4245,34 @@
         <v/>
       </c>
       <c r="D7" s="25">
-        <f>SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY())*(CashTransactions!B2:B500&lt;=TODAY())*(CashTransactions!D2:D500&gt;0)*CashTransactions!D2:D500)+SUMPRODUCT((DepositsData!F2:F100&gt;=TODAY())*(DepositsData!F2:F100&lt;=TODAY())*(DepositsData!G2:G100="Active")*(DepositsData!D2:D100+DepositsData!H2:H100))</f>
+        <f>LET(
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    depMaturity,DepositsData!F2:F100,
+    depPrincipal,DepositsData!D2:D100,
+    depInterest,DepositsData!H2:H100,
+    depStatus,DepositsData!G2:G100,
+    startDt,TODAY(),
+    endDt,TODAY(),
+    cashInflows,SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0),0)),
+    depositInflows,SUM(FILTER(depPrincipal+depInterest,(depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active"),0)),
+    cashInflows+depositInflows
+)</f>
         <v/>
       </c>
       <c r="E7" s="25">
-        <f>SUMPRODUCT((PaymentsData!B2:B500&gt;=TODAY())*(PaymentsData!B2:B500&lt;=TODAY())*(PaymentsData!F2:F500&lt;&gt;"Cancelled")*PaymentsData!D2:D500)+ABS(SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY())*(CashTransactions!B2:B500&lt;=TODAY())*(CashTransactions!D2:D500&lt;0)*CashTransactions!D2:D500))</f>
+        <f>LET(
+    payDates,PaymentsData!B2:B500,
+    payAmounts,PaymentsData!D2:D500,
+    payStatus,PaymentsData!F2:F500,
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    startDt,TODAY(),
+    endDt,TODAY(),
+    paymentOut,SUM(FILTER(payAmounts,(payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled"),0)),
+    cashOut,ABS(SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0),0))),
+    paymentOut+cashOut
+)</f>
         <v/>
       </c>
       <c r="F7" s="25">
@@ -3342,7 +4284,7 @@
         <v/>
       </c>
       <c r="H7" s="59">
-        <f>IFERROR(F7/C7,0)</f>
+        <f>LET(net,F7,start,C7,IFERROR(net/start,0))</f>
         <v/>
       </c>
     </row>
@@ -3357,11 +4299,34 @@
         <v/>
       </c>
       <c r="D8" s="25">
-        <f>SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY()-WEEKDAY(TODAY(),2)+1)*(CashTransactions!B2:B500&lt;=TODAY()-WEEKDAY(TODAY(),2)+7)*(CashTransactions!D2:D500&gt;0)*CashTransactions!D2:D500)+SUMPRODUCT((DepositsData!F2:F100&gt;=TODAY()-WEEKDAY(TODAY(),2)+1)*(DepositsData!F2:F100&lt;=TODAY()-WEEKDAY(TODAY(),2)+7)*(DepositsData!G2:G100="Active")*(DepositsData!D2:D100+DepositsData!H2:H100))</f>
+        <f>LET(
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    depMaturity,DepositsData!F2:F100,
+    depPrincipal,DepositsData!D2:D100,
+    depInterest,DepositsData!H2:H100,
+    depStatus,DepositsData!G2:G100,
+    startDt,TODAY()-WEEKDAY(TODAY(),2)+1,
+    endDt,TODAY()-WEEKDAY(TODAY(),2)+7,
+    cashInflows,SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0),0)),
+    depositInflows,SUM(FILTER(depPrincipal+depInterest,(depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active"),0)),
+    cashInflows+depositInflows
+)</f>
         <v/>
       </c>
       <c r="E8" s="25">
-        <f>SUMPRODUCT((PaymentsData!B2:B500&gt;=TODAY()-WEEKDAY(TODAY(),2)+1)*(PaymentsData!B2:B500&lt;=TODAY()-WEEKDAY(TODAY(),2)+7)*(PaymentsData!F2:F500&lt;&gt;"Cancelled")*PaymentsData!D2:D500)+ABS(SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY()-WEEKDAY(TODAY(),2)+1)*(CashTransactions!B2:B500&lt;=TODAY()-WEEKDAY(TODAY(),2)+7)*(CashTransactions!D2:D500&lt;0)*CashTransactions!D2:D500))</f>
+        <f>LET(
+    payDates,PaymentsData!B2:B500,
+    payAmounts,PaymentsData!D2:D500,
+    payStatus,PaymentsData!F2:F500,
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    startDt,TODAY()-WEEKDAY(TODAY(),2)+1,
+    endDt,TODAY()-WEEKDAY(TODAY(),2)+7,
+    paymentOut,SUM(FILTER(payAmounts,(payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled"),0)),
+    cashOut,ABS(SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0),0))),
+    paymentOut+cashOut
+)</f>
         <v/>
       </c>
       <c r="F8" s="25">
@@ -3373,7 +4338,7 @@
         <v/>
       </c>
       <c r="H8" s="59">
-        <f>IFERROR(F8/C8,0)</f>
+        <f>LET(net,F8,start,C8,IFERROR(net/start,0))</f>
         <v/>
       </c>
     </row>
@@ -3388,11 +4353,34 @@
         <v/>
       </c>
       <c r="D9" s="25">
-        <f>SUMPRODUCT((CashTransactions!B2:B500&gt;=DATE(YEAR(TODAY()),MONTH(TODAY()),1))*(CashTransactions!B2:B500&lt;=EOMONTH(TODAY(),0))*(CashTransactions!D2:D500&gt;0)*CashTransactions!D2:D500)+SUMPRODUCT((DepositsData!F2:F100&gt;=DATE(YEAR(TODAY()),MONTH(TODAY()),1))*(DepositsData!F2:F100&lt;=EOMONTH(TODAY(),0))*(DepositsData!G2:G100="Active")*(DepositsData!D2:D100+DepositsData!H2:H100))</f>
+        <f>LET(
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    depMaturity,DepositsData!F2:F100,
+    depPrincipal,DepositsData!D2:D100,
+    depInterest,DepositsData!H2:H100,
+    depStatus,DepositsData!G2:G100,
+    startDt,DATE(YEAR(TODAY()),MONTH(TODAY()),1),
+    endDt,EOMONTH(TODAY(),0),
+    cashInflows,SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0),0)),
+    depositInflows,SUM(FILTER(depPrincipal+depInterest,(depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active"),0)),
+    cashInflows+depositInflows
+)</f>
         <v/>
       </c>
       <c r="E9" s="25">
-        <f>SUMPRODUCT((PaymentsData!B2:B500&gt;=DATE(YEAR(TODAY()),MONTH(TODAY()),1))*(PaymentsData!B2:B500&lt;=EOMONTH(TODAY(),0))*(PaymentsData!F2:F500&lt;&gt;"Cancelled")*PaymentsData!D2:D500)+ABS(SUMPRODUCT((CashTransactions!B2:B500&gt;=DATE(YEAR(TODAY()),MONTH(TODAY()),1))*(CashTransactions!B2:B500&lt;=EOMONTH(TODAY(),0))*(CashTransactions!D2:D500&lt;0)*CashTransactions!D2:D500))</f>
+        <f>LET(
+    payDates,PaymentsData!B2:B500,
+    payAmounts,PaymentsData!D2:D500,
+    payStatus,PaymentsData!F2:F500,
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    startDt,DATE(YEAR(TODAY()),MONTH(TODAY()),1),
+    endDt,EOMONTH(TODAY(),0),
+    paymentOut,SUM(FILTER(payAmounts,(payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled"),0)),
+    cashOut,ABS(SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0),0))),
+    paymentOut+cashOut
+)</f>
         <v/>
       </c>
       <c r="F9" s="25">
@@ -3404,7 +4392,7 @@
         <v/>
       </c>
       <c r="H9" s="59">
-        <f>IFERROR(F9/C9,0)</f>
+        <f>LET(net,F9,start,C9,IFERROR(net/start,0))</f>
         <v/>
       </c>
     </row>
@@ -3419,11 +4407,34 @@
         <v/>
       </c>
       <c r="D10" s="25">
-        <f>SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY())*(CashTransactions!B2:B500&lt;=TODAY()+30)*(CashTransactions!D2:D500&gt;0)*CashTransactions!D2:D500)+SUMPRODUCT((DepositsData!F2:F100&gt;=TODAY())*(DepositsData!F2:F100&lt;=TODAY()+30)*(DepositsData!G2:G100="Active")*(DepositsData!D2:D100+DepositsData!H2:H100))</f>
+        <f>LET(
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    depMaturity,DepositsData!F2:F100,
+    depPrincipal,DepositsData!D2:D100,
+    depInterest,DepositsData!H2:H100,
+    depStatus,DepositsData!G2:G100,
+    startDt,TODAY(),
+    endDt,TODAY()+30,
+    cashInflows,SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0),0)),
+    depositInflows,SUM(FILTER(depPrincipal+depInterest,(depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active"),0)),
+    cashInflows+depositInflows
+)</f>
         <v/>
       </c>
       <c r="E10" s="25">
-        <f>SUMPRODUCT((PaymentsData!B2:B500&gt;=TODAY())*(PaymentsData!B2:B500&lt;=TODAY()+30)*(PaymentsData!F2:F500&lt;&gt;"Cancelled")*PaymentsData!D2:D500)+ABS(SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY())*(CashTransactions!B2:B500&lt;=TODAY()+30)*(CashTransactions!D2:D500&lt;0)*CashTransactions!D2:D500))</f>
+        <f>LET(
+    payDates,PaymentsData!B2:B500,
+    payAmounts,PaymentsData!D2:D500,
+    payStatus,PaymentsData!F2:F500,
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    startDt,TODAY(),
+    endDt,TODAY()+30,
+    paymentOut,SUM(FILTER(payAmounts,(payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled"),0)),
+    cashOut,ABS(SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0),0))),
+    paymentOut+cashOut
+)</f>
         <v/>
       </c>
       <c r="F10" s="25">
@@ -3435,7 +4446,7 @@
         <v/>
       </c>
       <c r="H10" s="59">
-        <f>IFERROR(F10/C10,0)</f>
+        <f>LET(net,F10,start,C10,IFERROR(net/start,0))</f>
         <v/>
       </c>
     </row>
@@ -3450,11 +4461,34 @@
         <v/>
       </c>
       <c r="D11" s="25">
-        <f>SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY())*(CashTransactions!B2:B500&lt;=TODAY()+60)*(CashTransactions!D2:D500&gt;0)*CashTransactions!D2:D500)+SUMPRODUCT((DepositsData!F2:F100&gt;=TODAY())*(DepositsData!F2:F100&lt;=TODAY()+60)*(DepositsData!G2:G100="Active")*(DepositsData!D2:D100+DepositsData!H2:H100))</f>
+        <f>LET(
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    depMaturity,DepositsData!F2:F100,
+    depPrincipal,DepositsData!D2:D100,
+    depInterest,DepositsData!H2:H100,
+    depStatus,DepositsData!G2:G100,
+    startDt,TODAY(),
+    endDt,TODAY()+60,
+    cashInflows,SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0),0)),
+    depositInflows,SUM(FILTER(depPrincipal+depInterest,(depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active"),0)),
+    cashInflows+depositInflows
+)</f>
         <v/>
       </c>
       <c r="E11" s="25">
-        <f>SUMPRODUCT((PaymentsData!B2:B500&gt;=TODAY())*(PaymentsData!B2:B500&lt;=TODAY()+60)*(PaymentsData!F2:F500&lt;&gt;"Cancelled")*PaymentsData!D2:D500)+ABS(SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY())*(CashTransactions!B2:B500&lt;=TODAY()+60)*(CashTransactions!D2:D500&lt;0)*CashTransactions!D2:D500))</f>
+        <f>LET(
+    payDates,PaymentsData!B2:B500,
+    payAmounts,PaymentsData!D2:D500,
+    payStatus,PaymentsData!F2:F500,
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    startDt,TODAY(),
+    endDt,TODAY()+60,
+    paymentOut,SUM(FILTER(payAmounts,(payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled"),0)),
+    cashOut,ABS(SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0),0))),
+    paymentOut+cashOut
+)</f>
         <v/>
       </c>
       <c r="F11" s="25">
@@ -3466,7 +4500,7 @@
         <v/>
       </c>
       <c r="H11" s="59">
-        <f>IFERROR(F11/C11,0)</f>
+        <f>LET(net,F11,start,C11,IFERROR(net/start,0))</f>
         <v/>
       </c>
     </row>
@@ -3481,11 +4515,34 @@
         <v/>
       </c>
       <c r="D12" s="25">
-        <f>SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY())*(CashTransactions!B2:B500&lt;=TODAY()+90)*(CashTransactions!D2:D500&gt;0)*CashTransactions!D2:D500)+SUMPRODUCT((DepositsData!F2:F100&gt;=TODAY())*(DepositsData!F2:F100&lt;=TODAY()+90)*(DepositsData!G2:G100="Active")*(DepositsData!D2:D100+DepositsData!H2:H100))</f>
+        <f>LET(
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    depMaturity,DepositsData!F2:F100,
+    depPrincipal,DepositsData!D2:D100,
+    depInterest,DepositsData!H2:H100,
+    depStatus,DepositsData!G2:G100,
+    startDt,TODAY(),
+    endDt,TODAY()+90,
+    cashInflows,SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0),0)),
+    depositInflows,SUM(FILTER(depPrincipal+depInterest,(depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active"),0)),
+    cashInflows+depositInflows
+)</f>
         <v/>
       </c>
       <c r="E12" s="25">
-        <f>SUMPRODUCT((PaymentsData!B2:B500&gt;=TODAY())*(PaymentsData!B2:B500&lt;=TODAY()+90)*(PaymentsData!F2:F500&lt;&gt;"Cancelled")*PaymentsData!D2:D500)+ABS(SUMPRODUCT((CashTransactions!B2:B500&gt;=TODAY())*(CashTransactions!B2:B500&lt;=TODAY()+90)*(CashTransactions!D2:D500&lt;0)*CashTransactions!D2:D500))</f>
+        <f>LET(
+    payDates,PaymentsData!B2:B500,
+    payAmounts,PaymentsData!D2:D500,
+    payStatus,PaymentsData!F2:F500,
+    txDates,CashTransactions!B2:B500,
+    txAmounts,CashTransactions!D2:D500,
+    startDt,TODAY(),
+    endDt,TODAY()+90,
+    paymentOut,SUM(FILTER(payAmounts,(payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled"),0)),
+    cashOut,ABS(SUM(FILTER(txAmounts,(txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0),0))),
+    paymentOut+cashOut
+)</f>
         <v/>
       </c>
       <c r="F12" s="25">
@@ -3497,7 +4554,7 @@
         <v/>
       </c>
       <c r="H12" s="59">
-        <f>IFERROR(F12/C12,0)</f>
+        <f>LET(net,F12,start,C12,IFERROR(net/start,0))</f>
         <v/>
       </c>
     </row>
@@ -3546,15 +4603,36 @@
         <v/>
       </c>
       <c r="C16" s="63">
-        <f>TEXT(B16,"dddd")</f>
+        <f>LET(dt,B16,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D16" s="64">
-        <f>SUMPRODUCT((CashTransactions!B:B=B16)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B16)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B16,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E16" s="64">
-        <f>SUMPRODUCT((PaymentsData!B:B=B16)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B16)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B16,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F16" s="64">
@@ -3572,15 +4650,36 @@
         <v/>
       </c>
       <c r="C17" s="21">
-        <f>TEXT(B17,"dddd")</f>
+        <f>LET(dt,B17,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D17" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B17)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B17)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B17,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E17" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B17)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B17)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B17,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F17" s="23">
@@ -3598,15 +4697,36 @@
         <v/>
       </c>
       <c r="C18" s="21">
-        <f>TEXT(B18,"dddd")</f>
+        <f>LET(dt,B18,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D18" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B18)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B18)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B18,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E18" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B18)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B18)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B18,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F18" s="23">
@@ -3624,15 +4744,36 @@
         <v/>
       </c>
       <c r="C19" s="21">
-        <f>TEXT(B19,"dddd")</f>
+        <f>LET(dt,B19,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D19" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B19)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B19)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B19,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E19" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B19)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B19)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B19,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F19" s="23">
@@ -3650,15 +4791,36 @@
         <v/>
       </c>
       <c r="C20" s="21">
-        <f>TEXT(B20,"dddd")</f>
+        <f>LET(dt,B20,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D20" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B20)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B20)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B20,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E20" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B20)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B20)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B20,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F20" s="23">
@@ -3676,15 +4838,36 @@
         <v/>
       </c>
       <c r="C21" s="21">
-        <f>TEXT(B21,"dddd")</f>
+        <f>LET(dt,B21,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D21" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B21)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B21)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B21,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E21" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B21)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B21)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B21,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F21" s="23">
@@ -3702,15 +4885,36 @@
         <v/>
       </c>
       <c r="C22" s="21">
-        <f>TEXT(B22,"dddd")</f>
+        <f>LET(dt,B22,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D22" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B22)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B22)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B22,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E22" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B22)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B22)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B22,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F22" s="23">
@@ -3728,15 +4932,36 @@
         <v/>
       </c>
       <c r="C23" s="21">
-        <f>TEXT(B23,"dddd")</f>
+        <f>LET(dt,B23,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D23" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B23)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B23)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B23,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E23" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B23)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B23)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B23,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F23" s="23">
@@ -3754,15 +4979,36 @@
         <v/>
       </c>
       <c r="C24" s="21">
-        <f>TEXT(B24,"dddd")</f>
+        <f>LET(dt,B24,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D24" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B24)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B24)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B24,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E24" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B24)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B24)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B24,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F24" s="23">
@@ -3780,15 +5026,36 @@
         <v/>
       </c>
       <c r="C25" s="21">
-        <f>TEXT(B25,"dddd")</f>
+        <f>LET(dt,B25,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D25" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B25)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B25)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B25,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E25" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B25)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B25)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B25,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F25" s="23">
@@ -3806,15 +5073,36 @@
         <v/>
       </c>
       <c r="C26" s="21">
-        <f>TEXT(B26,"dddd")</f>
+        <f>LET(dt,B26,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D26" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B26)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B26)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B26,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E26" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B26)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B26)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B26,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F26" s="23">
@@ -3832,15 +5120,36 @@
         <v/>
       </c>
       <c r="C27" s="21">
-        <f>TEXT(B27,"dddd")</f>
+        <f>LET(dt,B27,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D27" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B27)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B27)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B27,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E27" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B27)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B27)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B27,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F27" s="23">
@@ -3858,15 +5167,36 @@
         <v/>
       </c>
       <c r="C28" s="21">
-        <f>TEXT(B28,"dddd")</f>
+        <f>LET(dt,B28,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D28" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B28)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B28)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B28,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E28" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B28)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B28)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B28,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F28" s="23">
@@ -3884,15 +5214,36 @@
         <v/>
       </c>
       <c r="C29" s="21">
-        <f>TEXT(B29,"dddd")</f>
+        <f>LET(dt,B29,TEXT(dt,"dddd"))</f>
         <v/>
       </c>
       <c r="D29" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B=B29)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F=B29)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    dt,B29,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMIF(txDates,dt,txAmounts),
+    depIn,SUMPRODUCT((depMaturity=dt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    MAX(0,cashIn)+depIn
+)</f>
         <v/>
       </c>
       <c r="E29" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B=B29)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B=B29)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    dt,B29,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates=dt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(MIN(0,SUMIF(txDates,dt,txAmounts))),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F29" s="23">
@@ -3953,11 +5304,34 @@
         <v/>
       </c>
       <c r="D34" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B&gt;=B34)*(CashTransactions!B:B&lt;=B34+6)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F&gt;=B34)*(DepositsData!F:F&lt;=B34+6)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    startDt,B34,
+    endDt,B34+6,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0)*txAmounts),
+    depIn,SUMPRODUCT((depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    cashIn+depIn
+)</f>
         <v/>
       </c>
       <c r="E34" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B&gt;=B34)*(PaymentsData!B:B&lt;=B34+6)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B&gt;=B34)*(CashTransactions!B:B&lt;=B34+6)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    startDt,B34,
+    endDt,B34+6,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0)*txAmounts)),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F34" s="23">
@@ -3979,11 +5353,34 @@
         <v/>
       </c>
       <c r="D35" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B&gt;=B35)*(CashTransactions!B:B&lt;=B35+6)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F&gt;=B35)*(DepositsData!F:F&lt;=B35+6)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    startDt,B35,
+    endDt,B35+6,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0)*txAmounts),
+    depIn,SUMPRODUCT((depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    cashIn+depIn
+)</f>
         <v/>
       </c>
       <c r="E35" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B&gt;=B35)*(PaymentsData!B:B&lt;=B35+6)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B&gt;=B35)*(CashTransactions!B:B&lt;=B35+6)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    startDt,B35,
+    endDt,B35+6,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0)*txAmounts)),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F35" s="23">
@@ -4005,11 +5402,34 @@
         <v/>
       </c>
       <c r="D36" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B&gt;=B36)*(CashTransactions!B:B&lt;=B36+6)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F&gt;=B36)*(DepositsData!F:F&lt;=B36+6)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    startDt,B36,
+    endDt,B36+6,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0)*txAmounts),
+    depIn,SUMPRODUCT((depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    cashIn+depIn
+)</f>
         <v/>
       </c>
       <c r="E36" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B&gt;=B36)*(PaymentsData!B:B&lt;=B36+6)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B&gt;=B36)*(CashTransactions!B:B&lt;=B36+6)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    startDt,B36,
+    endDt,B36+6,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0)*txAmounts)),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F36" s="23">
@@ -4031,11 +5451,34 @@
         <v/>
       </c>
       <c r="D37" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B&gt;=B37)*(CashTransactions!B:B&lt;=B37+6)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F&gt;=B37)*(DepositsData!F:F&lt;=B37+6)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    startDt,B37,
+    endDt,B37+6,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0)*txAmounts),
+    depIn,SUMPRODUCT((depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    cashIn+depIn
+)</f>
         <v/>
       </c>
       <c r="E37" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B&gt;=B37)*(PaymentsData!B:B&lt;=B37+6)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B&gt;=B37)*(CashTransactions!B:B&lt;=B37+6)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    startDt,B37,
+    endDt,B37+6,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0)*txAmounts)),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F37" s="23">
@@ -4057,11 +5500,34 @@
         <v/>
       </c>
       <c r="D38" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B&gt;=B38)*(CashTransactions!B:B&lt;=B38+6)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F&gt;=B38)*(DepositsData!F:F&lt;=B38+6)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    startDt,B38,
+    endDt,B38+6,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0)*txAmounts),
+    depIn,SUMPRODUCT((depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    cashIn+depIn
+)</f>
         <v/>
       </c>
       <c r="E38" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B&gt;=B38)*(PaymentsData!B:B&lt;=B38+6)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B&gt;=B38)*(CashTransactions!B:B&lt;=B38+6)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    startDt,B38,
+    endDt,B38+6,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0)*txAmounts)),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F38" s="23">
@@ -4083,11 +5549,34 @@
         <v/>
       </c>
       <c r="D39" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B&gt;=B39)*(CashTransactions!B:B&lt;=B39+6)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F&gt;=B39)*(DepositsData!F:F&lt;=B39+6)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    startDt,B39,
+    endDt,B39+6,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0)*txAmounts),
+    depIn,SUMPRODUCT((depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    cashIn+depIn
+)</f>
         <v/>
       </c>
       <c r="E39" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B&gt;=B39)*(PaymentsData!B:B&lt;=B39+6)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B&gt;=B39)*(CashTransactions!B:B&lt;=B39+6)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    startDt,B39,
+    endDt,B39+6,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0)*txAmounts)),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F39" s="23">
@@ -4109,11 +5598,34 @@
         <v/>
       </c>
       <c r="D40" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B&gt;=B40)*(CashTransactions!B:B&lt;=B40+6)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F&gt;=B40)*(DepositsData!F:F&lt;=B40+6)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    startDt,B40,
+    endDt,B40+6,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0)*txAmounts),
+    depIn,SUMPRODUCT((depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    cashIn+depIn
+)</f>
         <v/>
       </c>
       <c r="E40" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B&gt;=B40)*(PaymentsData!B:B&lt;=B40+6)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B&gt;=B40)*(CashTransactions!B:B&lt;=B40+6)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    startDt,B40,
+    endDt,B40+6,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0)*txAmounts)),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F40" s="23">
@@ -4135,11 +5647,34 @@
         <v/>
       </c>
       <c r="D41" s="23">
-        <f>SUMPRODUCT((CashTransactions!B:B&gt;=B41)*(CashTransactions!B:B&lt;=B41+6)*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)+SUMPRODUCT((DepositsData!F:F&gt;=B41)*(DepositsData!F:F&lt;=B41+6)*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    startDt,B41,
+    endDt,B41+6,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    cashIn,SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&gt;0)*txAmounts),
+    depIn,SUMPRODUCT((depMaturity&gt;=startDt)*(depMaturity&lt;=endDt)*(depStatus="Active")*(depPrincipal+depInterest)),
+    cashIn+depIn
+)</f>
         <v/>
       </c>
       <c r="E41" s="23">
-        <f>SUMPRODUCT((PaymentsData!B:B&gt;=B41)*(PaymentsData!B:B&lt;=B41+6)*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)+ABS(SUMPRODUCT((CashTransactions!B:B&gt;=B41)*(CashTransactions!B:B&lt;=B41+6)*(CashTransactions!D:D&lt;0)*CashTransactions!D:D))</f>
+        <f>LET(
+    startDt,B41,
+    endDt,B41+6,
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    payments,SUMPRODUCT((payDates&gt;=startDt)*(payDates&lt;=endDt)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    cashOut,ABS(SUMPRODUCT((txDates&gt;=startDt)*(txDates&lt;=endDt)*(txAmounts&lt;0)*txAmounts)),
+    payments+cashOut
+)</f>
         <v/>
       </c>
       <c r="F41" s="23">
@@ -4196,11 +5731,26 @@
         <v/>
       </c>
       <c r="C46" s="23">
-        <f>SUMPRODUCT((MONTH(CashTransactions!B:B)=MONTH(EOMONTH(TODAY(),0)))*(YEAR(CashTransactions!B:B)=YEAR(EOMONTH(TODAY(),0)))*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),0)),
+    targetYear,YEAR(EOMONTH(TODAY(),0)),
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    cashIn,SUMPRODUCT((MONTH(txDates)=targetMonth)*(YEAR(txDates)=targetYear)*(txAmounts&gt;0)*txAmounts),
+    cashIn
+)</f>
         <v/>
       </c>
       <c r="D46" s="23">
-        <f>SUMPRODUCT((MONTH(PaymentsData!B:B)=MONTH(EOMONTH(TODAY(),0)))*(YEAR(PaymentsData!B:B)=YEAR(EOMONTH(TODAY(),0)))*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),0)),
+    targetYear,YEAR(EOMONTH(TODAY(),0)),
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    payments,SUMPRODUCT((MONTH(payDates)=targetMonth)*(YEAR(payDates)=targetYear)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    payments
+)</f>
         <v/>
       </c>
       <c r="E46" s="23">
@@ -4212,7 +5762,15 @@
         <v/>
       </c>
       <c r="G46" s="23">
-        <f>SUMPRODUCT((MONTH(DepositsData!F:F)=MONTH(EOMONTH(TODAY(),0)))*(YEAR(DepositsData!F:F)=YEAR(EOMONTH(TODAY(),0)))*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),0)),
+    targetYear,YEAR(EOMONTH(TODAY(),0)),
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    SUMPRODUCT((MONTH(depMaturity)=targetMonth)*(YEAR(depMaturity)=targetYear)*(depStatus="Active")*(depPrincipal+depInterest))
+)</f>
         <v/>
       </c>
     </row>
@@ -4222,11 +5780,26 @@
         <v/>
       </c>
       <c r="C47" s="23">
-        <f>SUMPRODUCT((MONTH(CashTransactions!B:B)=MONTH(EOMONTH(TODAY(),1)))*(YEAR(CashTransactions!B:B)=YEAR(EOMONTH(TODAY(),1)))*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),1)),
+    targetYear,YEAR(EOMONTH(TODAY(),1)),
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    cashIn,SUMPRODUCT((MONTH(txDates)=targetMonth)*(YEAR(txDates)=targetYear)*(txAmounts&gt;0)*txAmounts),
+    cashIn
+)</f>
         <v/>
       </c>
       <c r="D47" s="23">
-        <f>SUMPRODUCT((MONTH(PaymentsData!B:B)=MONTH(EOMONTH(TODAY(),1)))*(YEAR(PaymentsData!B:B)=YEAR(EOMONTH(TODAY(),1)))*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),1)),
+    targetYear,YEAR(EOMONTH(TODAY(),1)),
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    payments,SUMPRODUCT((MONTH(payDates)=targetMonth)*(YEAR(payDates)=targetYear)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    payments
+)</f>
         <v/>
       </c>
       <c r="E47" s="23">
@@ -4238,7 +5811,15 @@
         <v/>
       </c>
       <c r="G47" s="23">
-        <f>SUMPRODUCT((MONTH(DepositsData!F:F)=MONTH(EOMONTH(TODAY(),1)))*(YEAR(DepositsData!F:F)=YEAR(EOMONTH(TODAY(),1)))*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),1)),
+    targetYear,YEAR(EOMONTH(TODAY(),1)),
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    SUMPRODUCT((MONTH(depMaturity)=targetMonth)*(YEAR(depMaturity)=targetYear)*(depStatus="Active")*(depPrincipal+depInterest))
+)</f>
         <v/>
       </c>
     </row>
@@ -4248,11 +5829,26 @@
         <v/>
       </c>
       <c r="C48" s="23">
-        <f>SUMPRODUCT((MONTH(CashTransactions!B:B)=MONTH(EOMONTH(TODAY(),2)))*(YEAR(CashTransactions!B:B)=YEAR(EOMONTH(TODAY(),2)))*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),2)),
+    targetYear,YEAR(EOMONTH(TODAY(),2)),
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    cashIn,SUMPRODUCT((MONTH(txDates)=targetMonth)*(YEAR(txDates)=targetYear)*(txAmounts&gt;0)*txAmounts),
+    cashIn
+)</f>
         <v/>
       </c>
       <c r="D48" s="23">
-        <f>SUMPRODUCT((MONTH(PaymentsData!B:B)=MONTH(EOMONTH(TODAY(),2)))*(YEAR(PaymentsData!B:B)=YEAR(EOMONTH(TODAY(),2)))*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),2)),
+    targetYear,YEAR(EOMONTH(TODAY(),2)),
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    payments,SUMPRODUCT((MONTH(payDates)=targetMonth)*(YEAR(payDates)=targetYear)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    payments
+)</f>
         <v/>
       </c>
       <c r="E48" s="23">
@@ -4264,7 +5860,15 @@
         <v/>
       </c>
       <c r="G48" s="23">
-        <f>SUMPRODUCT((MONTH(DepositsData!F:F)=MONTH(EOMONTH(TODAY(),2)))*(YEAR(DepositsData!F:F)=YEAR(EOMONTH(TODAY(),2)))*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),2)),
+    targetYear,YEAR(EOMONTH(TODAY(),2)),
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    SUMPRODUCT((MONTH(depMaturity)=targetMonth)*(YEAR(depMaturity)=targetYear)*(depStatus="Active")*(depPrincipal+depInterest))
+)</f>
         <v/>
       </c>
     </row>
@@ -4274,11 +5878,26 @@
         <v/>
       </c>
       <c r="C49" s="23">
-        <f>SUMPRODUCT((MONTH(CashTransactions!B:B)=MONTH(EOMONTH(TODAY(),3)))*(YEAR(CashTransactions!B:B)=YEAR(EOMONTH(TODAY(),3)))*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),3)),
+    targetYear,YEAR(EOMONTH(TODAY(),3)),
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    cashIn,SUMPRODUCT((MONTH(txDates)=targetMonth)*(YEAR(txDates)=targetYear)*(txAmounts&gt;0)*txAmounts),
+    cashIn
+)</f>
         <v/>
       </c>
       <c r="D49" s="23">
-        <f>SUMPRODUCT((MONTH(PaymentsData!B:B)=MONTH(EOMONTH(TODAY(),3)))*(YEAR(PaymentsData!B:B)=YEAR(EOMONTH(TODAY(),3)))*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),3)),
+    targetYear,YEAR(EOMONTH(TODAY(),3)),
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    payments,SUMPRODUCT((MONTH(payDates)=targetMonth)*(YEAR(payDates)=targetYear)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    payments
+)</f>
         <v/>
       </c>
       <c r="E49" s="23">
@@ -4290,7 +5909,15 @@
         <v/>
       </c>
       <c r="G49" s="23">
-        <f>SUMPRODUCT((MONTH(DepositsData!F:F)=MONTH(EOMONTH(TODAY(),3)))*(YEAR(DepositsData!F:F)=YEAR(EOMONTH(TODAY(),3)))*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),3)),
+    targetYear,YEAR(EOMONTH(TODAY(),3)),
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    SUMPRODUCT((MONTH(depMaturity)=targetMonth)*(YEAR(depMaturity)=targetYear)*(depStatus="Active")*(depPrincipal+depInterest))
+)</f>
         <v/>
       </c>
     </row>
@@ -4300,11 +5927,26 @@
         <v/>
       </c>
       <c r="C50" s="23">
-        <f>SUMPRODUCT((MONTH(CashTransactions!B:B)=MONTH(EOMONTH(TODAY(),4)))*(YEAR(CashTransactions!B:B)=YEAR(EOMONTH(TODAY(),4)))*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),4)),
+    targetYear,YEAR(EOMONTH(TODAY(),4)),
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    cashIn,SUMPRODUCT((MONTH(txDates)=targetMonth)*(YEAR(txDates)=targetYear)*(txAmounts&gt;0)*txAmounts),
+    cashIn
+)</f>
         <v/>
       </c>
       <c r="D50" s="23">
-        <f>SUMPRODUCT((MONTH(PaymentsData!B:B)=MONTH(EOMONTH(TODAY(),4)))*(YEAR(PaymentsData!B:B)=YEAR(EOMONTH(TODAY(),4)))*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),4)),
+    targetYear,YEAR(EOMONTH(TODAY(),4)),
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    payments,SUMPRODUCT((MONTH(payDates)=targetMonth)*(YEAR(payDates)=targetYear)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    payments
+)</f>
         <v/>
       </c>
       <c r="E50" s="23">
@@ -4316,7 +5958,15 @@
         <v/>
       </c>
       <c r="G50" s="23">
-        <f>SUMPRODUCT((MONTH(DepositsData!F:F)=MONTH(EOMONTH(TODAY(),4)))*(YEAR(DepositsData!F:F)=YEAR(EOMONTH(TODAY(),4)))*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),4)),
+    targetYear,YEAR(EOMONTH(TODAY(),4)),
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    SUMPRODUCT((MONTH(depMaturity)=targetMonth)*(YEAR(depMaturity)=targetYear)*(depStatus="Active")*(depPrincipal+depInterest))
+)</f>
         <v/>
       </c>
     </row>
@@ -4326,11 +5976,26 @@
         <v/>
       </c>
       <c r="C51" s="23">
-        <f>SUMPRODUCT((MONTH(CashTransactions!B:B)=MONTH(EOMONTH(TODAY(),5)))*(YEAR(CashTransactions!B:B)=YEAR(EOMONTH(TODAY(),5)))*(CashTransactions!D:D&gt;0)*CashTransactions!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),5)),
+    targetYear,YEAR(EOMONTH(TODAY(),5)),
+    txDates,CashTransactions!B:B,
+    txAmounts,CashTransactions!D:D,
+    cashIn,SUMPRODUCT((MONTH(txDates)=targetMonth)*(YEAR(txDates)=targetYear)*(txAmounts&gt;0)*txAmounts),
+    cashIn
+)</f>
         <v/>
       </c>
       <c r="D51" s="23">
-        <f>SUMPRODUCT((MONTH(PaymentsData!B:B)=MONTH(EOMONTH(TODAY(),5)))*(YEAR(PaymentsData!B:B)=YEAR(EOMONTH(TODAY(),5)))*(PaymentsData!F:F&lt;&gt;"Cancelled")*PaymentsData!D:D)</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),5)),
+    targetYear,YEAR(EOMONTH(TODAY(),5)),
+    payDates,PaymentsData!B:B,
+    payAmounts,PaymentsData!D:D,
+    payStatus,PaymentsData!F:F,
+    payments,SUMPRODUCT((MONTH(payDates)=targetMonth)*(YEAR(payDates)=targetYear)*(payStatus&lt;&gt;"Cancelled")*payAmounts),
+    payments
+)</f>
         <v/>
       </c>
       <c r="E51" s="23">
@@ -4342,7 +6007,15 @@
         <v/>
       </c>
       <c r="G51" s="23">
-        <f>SUMPRODUCT((MONTH(DepositsData!F:F)=MONTH(EOMONTH(TODAY(),5)))*(YEAR(DepositsData!F:F)=YEAR(EOMONTH(TODAY(),5)))*(DepositsData!G:G="Active")*(DepositsData!D:D+DepositsData!H:H))</f>
+        <f>LET(
+    targetMonth,MONTH(EOMONTH(TODAY(),5)),
+    targetYear,YEAR(EOMONTH(TODAY(),5)),
+    depMaturity,DepositsData!F:F,
+    depPrincipal,DepositsData!D:D,
+    depInterest,DepositsData!H:H,
+    depStatus,DepositsData!G:G,
+    SUMPRODUCT((MONTH(depMaturity)=targetMonth)*(YEAR(depMaturity)=targetYear)*(depStatus="Active")*(depPrincipal+depInterest))
+)</f>
         <v/>
       </c>
     </row>
@@ -4357,76 +6030,6 @@
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>F7&lt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B16:G16">
-    <cfRule type="expression" priority="3" dxfId="4">
-      <formula>OR(WEEKDAY(B16)=1,WEEKDAY(B16)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B17:G17">
-    <cfRule type="expression" priority="4" dxfId="4">
-      <formula>OR(WEEKDAY(B17)=1,WEEKDAY(B17)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B18:G18">
-    <cfRule type="expression" priority="5" dxfId="4">
-      <formula>OR(WEEKDAY(B18)=1,WEEKDAY(B18)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B19:G19">
-    <cfRule type="expression" priority="6" dxfId="4">
-      <formula>OR(WEEKDAY(B19)=1,WEEKDAY(B19)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B20:G20">
-    <cfRule type="expression" priority="7" dxfId="4">
-      <formula>OR(WEEKDAY(B20)=1,WEEKDAY(B20)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B21:G21">
-    <cfRule type="expression" priority="8" dxfId="4">
-      <formula>OR(WEEKDAY(B21)=1,WEEKDAY(B21)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B22:G22">
-    <cfRule type="expression" priority="9" dxfId="4">
-      <formula>OR(WEEKDAY(B22)=1,WEEKDAY(B22)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B23:G23">
-    <cfRule type="expression" priority="10" dxfId="4">
-      <formula>OR(WEEKDAY(B23)=1,WEEKDAY(B23)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B24:G24">
-    <cfRule type="expression" priority="11" dxfId="4">
-      <formula>OR(WEEKDAY(B24)=1,WEEKDAY(B24)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B25:G25">
-    <cfRule type="expression" priority="12" dxfId="4">
-      <formula>OR(WEEKDAY(B25)=1,WEEKDAY(B25)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B26:G26">
-    <cfRule type="expression" priority="13" dxfId="4">
-      <formula>OR(WEEKDAY(B26)=1,WEEKDAY(B26)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B27:G27">
-    <cfRule type="expression" priority="14" dxfId="4">
-      <formula>OR(WEEKDAY(B27)=1,WEEKDAY(B27)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B28:G28">
-    <cfRule type="expression" priority="15" dxfId="4">
-      <formula>OR(WEEKDAY(B28)=1,WEEKDAY(B28)=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B29:G29">
-    <cfRule type="expression" priority="16" dxfId="4">
-      <formula>OR(WEEKDAY(B29)=1,WEEKDAY(B29)=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4495,7 +6098,7 @@
         </is>
       </c>
       <c r="B2" s="67" t="n">
-        <v>46005.70098003133</v>
+        <v>46005.70604491312</v>
       </c>
       <c r="C2" s="21" t="inlineStr">
         <is>
@@ -4528,7 +6131,7 @@
         </is>
       </c>
       <c r="B3" s="67" t="n">
-        <v>46008.70098003146</v>
+        <v>46008.70604491318</v>
       </c>
       <c r="C3" s="21" t="inlineStr">
         <is>
@@ -4561,7 +6164,7 @@
         </is>
       </c>
       <c r="B4" s="67" t="n">
-        <v>46010.70098003147</v>
+        <v>46010.7060449132</v>
       </c>
       <c r="C4" s="21" t="inlineStr">
         <is>
@@ -4594,7 +6197,7 @@
         </is>
       </c>
       <c r="B5" s="67" t="n">
-        <v>46013.70098003148</v>
+        <v>46013.7060449132</v>
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
@@ -4627,7 +6230,7 @@
         </is>
       </c>
       <c r="B6" s="67" t="n">
-        <v>46015.70098003149</v>
+        <v>46015.70604491322</v>
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
@@ -4660,7 +6263,7 @@
         </is>
       </c>
       <c r="B7" s="67" t="n">
-        <v>46018.70098003151</v>
+        <v>46018.70604491323</v>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
@@ -4693,7 +6296,7 @@
         </is>
       </c>
       <c r="B8" s="67" t="n">
-        <v>46021.70098003151</v>
+        <v>46021.70604491324</v>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
@@ -4726,7 +6329,7 @@
         </is>
       </c>
       <c r="B9" s="67" t="n">
-        <v>46023.70098003153</v>
+        <v>46023.70604491326</v>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
@@ -4759,7 +6362,7 @@
         </is>
       </c>
       <c r="B10" s="67" t="n">
-        <v>46000.70098003154</v>
+        <v>46000.70604491326</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -4792,7 +6395,7 @@
         </is>
       </c>
       <c r="B11" s="67" t="n">
-        <v>45998.70098003155</v>
+        <v>45998.70604491328</v>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
@@ -4825,7 +6428,7 @@
         </is>
       </c>
       <c r="B12" s="67" t="n">
-        <v>46028.70098003156</v>
+        <v>46028.70604491328</v>
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
@@ -4858,7 +6461,7 @@
         </is>
       </c>
       <c r="B13" s="67" t="n">
-        <v>46031.70098003157</v>
+        <v>46031.7060449133</v>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
@@ -4987,7 +6590,7 @@
         </is>
       </c>
       <c r="C2" s="67" t="n">
-        <v>45913.7009800697</v>
+        <v>45913.70604494948</v>
       </c>
       <c r="D2" s="22" t="n">
         <v>500000</v>
@@ -4996,7 +6599,7 @@
         <v>0.045</v>
       </c>
       <c r="F2" s="67" t="n">
-        <v>46093.70098006978</v>
+        <v>46093.70604494954</v>
       </c>
       <c r="G2" s="21" t="inlineStr">
         <is>
@@ -5004,7 +6607,7 @@
         </is>
       </c>
       <c r="H2" s="22">
-        <f>D2*E2*(F2-C2)/365</f>
+        <f>LET(p,D2,r,E2,start,C2,maturity,F2,days,maturity-start,p*r*days/365)</f>
         <v/>
       </c>
       <c r="I2" s="21" t="inlineStr">
@@ -5025,7 +6628,7 @@
         </is>
       </c>
       <c r="C3" s="67" t="n">
-        <v>45943.70098006979</v>
+        <v>45943.70604494955</v>
       </c>
       <c r="D3" s="22" t="n">
         <v>250000</v>
@@ -5034,7 +6637,7 @@
         <v>0.0425</v>
       </c>
       <c r="F3" s="67" t="n">
-        <v>46123.7009800698</v>
+        <v>46123.70604494956</v>
       </c>
       <c r="G3" s="21" t="inlineStr">
         <is>
@@ -5042,7 +6645,7 @@
         </is>
       </c>
       <c r="H3" s="22">
-        <f>D3*E3*(F3-C3)/365</f>
+        <f>LET(p,D3,r,E3,start,C3,maturity,F3,days,maturity-start,p*r*days/365)</f>
         <v/>
       </c>
       <c r="I3" s="21" t="inlineStr">
@@ -5063,7 +6666,7 @@
         </is>
       </c>
       <c r="C4" s="67" t="n">
-        <v>45973.70098006981</v>
+        <v>45973.70604494957</v>
       </c>
       <c r="D4" s="22" t="n">
         <v>750000</v>
@@ -5072,7 +6675,7 @@
         <v>0.05</v>
       </c>
       <c r="F4" s="67" t="n">
-        <v>46338.70098006981</v>
+        <v>46338.70604494958</v>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
@@ -5080,7 +6683,7 @@
         </is>
       </c>
       <c r="H4" s="22">
-        <f>D4*E4*(F4-C4)/365</f>
+        <f>LET(p,D4,r,E4,start,C4,maturity,F4,days,maturity-start,p*r*days/365)</f>
         <v/>
       </c>
       <c r="I4" s="21" t="inlineStr">
@@ -5101,7 +6704,7 @@
         </is>
       </c>
       <c r="C5" s="67" t="n">
-        <v>45823.70098006986</v>
+        <v>45823.7060449496</v>
       </c>
       <c r="D5" s="22" t="n">
         <v>300000</v>
@@ -5110,7 +6713,7 @@
         <v>0.04</v>
       </c>
       <c r="F5" s="67" t="n">
-        <v>46008.70098006987</v>
+        <v>46008.7060449496</v>
       </c>
       <c r="G5" s="21" t="inlineStr">
         <is>
@@ -5118,7 +6721,7 @@
         </is>
       </c>
       <c r="H5" s="22">
-        <f>D5*E5*(F5-C5)/365</f>
+        <f>LET(p,D5,r,E5,start,C5,maturity,F5,days,maturity-start,p*r*days/365)</f>
         <v/>
       </c>
       <c r="I5" s="21" t="inlineStr">
@@ -5139,7 +6742,7 @@
         </is>
       </c>
       <c r="C6" s="67" t="n">
-        <v>45883.70098006989</v>
+        <v>45883.70604494961</v>
       </c>
       <c r="D6" s="22" t="n">
         <v>400000</v>
@@ -5148,7 +6751,7 @@
         <v>0.0475</v>
       </c>
       <c r="F6" s="67" t="n">
-        <v>46063.70098006989</v>
+        <v>46063.70604494962</v>
       </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
@@ -5156,7 +6759,7 @@
         </is>
       </c>
       <c r="H6" s="22">
-        <f>D6*E6*(F6-C6)/365</f>
+        <f>LET(p,D6,r,E6,start,C6,maturity,F6,days,maturity-start,p*r*days/365)</f>
         <v/>
       </c>
       <c r="I6" s="21" t="inlineStr">
@@ -5177,7 +6780,7 @@
         </is>
       </c>
       <c r="C7" s="67" t="n">
-        <v>45638.70098006989</v>
+        <v>45638.70604494963</v>
       </c>
       <c r="D7" s="22" t="n">
         <v>200000</v>
@@ -5186,7 +6789,7 @@
         <v>0.035</v>
       </c>
       <c r="F7" s="67" t="n">
-        <v>45998.70098006991</v>
+        <v>45998.70604494964</v>
       </c>
       <c r="G7" s="21" t="inlineStr">
         <is>
@@ -5194,7 +6797,7 @@
         </is>
       </c>
       <c r="H7" s="22">
-        <f>D7*E7*(F7-C7)/365</f>
+        <f>LET(p,D7,r,E7,start,C7,maturity,F7,days,maturity-start,p*r*days/365)</f>
         <v/>
       </c>
       <c r="I7" s="21" t="inlineStr">
@@ -5215,7 +6818,7 @@
         </is>
       </c>
       <c r="C8" s="67" t="n">
-        <v>45958.70098006992</v>
+        <v>45958.70604494964</v>
       </c>
       <c r="D8" s="22" t="n">
         <v>600000</v>
@@ -5224,7 +6827,7 @@
         <v>0.0525</v>
       </c>
       <c r="F8" s="67" t="n">
-        <v>46138.70098006993</v>
+        <v>46138.70604494965</v>
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
@@ -5232,7 +6835,7 @@
         </is>
       </c>
       <c r="H8" s="22">
-        <f>D8*E8*(F8-C8)/365</f>
+        <f>LET(p,D8,r,E8,start,C8,maturity,F8,days,maturity-start,p*r*days/365)</f>
         <v/>
       </c>
       <c r="I8" s="21" t="inlineStr">
@@ -5253,7 +6856,7 @@
         </is>
       </c>
       <c r="C9" s="67" t="n">
-        <v>45988.70098006993</v>
+        <v>45988.70604494966</v>
       </c>
       <c r="D9" s="22" t="n">
         <v>350000</v>
@@ -5262,7 +6865,7 @@
         <v>0.048</v>
       </c>
       <c r="F9" s="67" t="n">
-        <v>46168.70098006995</v>
+        <v>46168.70604494968</v>
       </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
@@ -5270,7 +6873,7 @@
         </is>
       </c>
       <c r="H9" s="22">
-        <f>D9*E9*(F9-C9)/365</f>
+        <f>LET(p,D9,r,E9,start,C9,maturity,F9,days,maturity-start,p*r*days/365)</f>
         <v/>
       </c>
       <c r="I9" s="21" t="inlineStr">
@@ -5369,7 +6972,7 @@
         </is>
       </c>
       <c r="B2" s="67" t="n">
-        <v>45993.70098010181</v>
+        <v>45993.70604498234</v>
       </c>
       <c r="C2" s="21" t="inlineStr">
         <is>
@@ -5411,7 +7014,7 @@
         </is>
       </c>
       <c r="B3" s="67" t="n">
-        <v>45994.70098010187</v>
+        <v>45994.7060449824</v>
       </c>
       <c r="C3" s="21" t="inlineStr">
         <is>
@@ -5453,7 +7056,7 @@
         </is>
       </c>
       <c r="B4" s="67" t="n">
-        <v>45995.70098010189</v>
+        <v>45995.7060449824</v>
       </c>
       <c r="C4" s="21" t="inlineStr">
         <is>
@@ -5495,7 +7098,7 @@
         </is>
       </c>
       <c r="B5" s="67" t="n">
-        <v>45996.70098010189</v>
+        <v>45996.70604498241</v>
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
@@ -5541,7 +7144,7 @@
         </is>
       </c>
       <c r="B6" s="67" t="n">
-        <v>45998.70098010193</v>
+        <v>45998.70604498242</v>
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
@@ -5583,7 +7186,7 @@
         </is>
       </c>
       <c r="B7" s="67" t="n">
-        <v>45999.70098010194</v>
+        <v>45999.70604498243</v>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
@@ -5629,7 +7232,7 @@
         </is>
       </c>
       <c r="B8" s="67" t="n">
-        <v>46000.70098010196</v>
+        <v>46000.70604498244</v>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
@@ -5675,7 +7278,7 @@
         </is>
       </c>
       <c r="B9" s="67" t="n">
-        <v>46001.70098010196</v>
+        <v>46001.70604498246</v>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
@@ -5721,7 +7324,7 @@
         </is>
       </c>
       <c r="B10" s="67" t="n">
-        <v>46002.70098010197</v>
+        <v>46002.70604498246</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -5763,7 +7366,7 @@
         </is>
       </c>
       <c r="B11" s="67" t="n">
-        <v>46003.70098010198</v>
+        <v>46003.70604498248</v>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
@@ -5804,10 +7407,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D500">
-    <cfRule type="expression" priority="1" dxfId="5">
+    <cfRule type="expression" priority="1" dxfId="4">
       <formula>D2&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="6">
+    <cfRule type="expression" priority="2" dxfId="5">
       <formula>D2&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5826,7 +7429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E25"/>
+  <dimension ref="B2:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -6075,6 +7678,85 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Modern Formula Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="75" t="inlineStr">
+        <is>
+          <t>LET</t>
+        </is>
+      </c>
+      <c r="C29" s="74" t="inlineStr">
+        <is>
+          <t>Defines named variables within formulas for clarity</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="75" t="inlineStr">
+        <is>
+          <t>FILTER</t>
+        </is>
+      </c>
+      <c r="C30" s="74" t="inlineStr">
+        <is>
+          <t>Returns array of values that meet criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="75" t="inlineStr">
+        <is>
+          <t>XLOOKUP</t>
+        </is>
+      </c>
+      <c r="C31" s="74" t="inlineStr">
+        <is>
+          <t>Modern replacement for VLOOKUP/INDEX-MATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="75" t="inlineStr">
+        <is>
+          <t>SORT</t>
+        </is>
+      </c>
+      <c r="C32" s="74" t="inlineStr">
+        <is>
+          <t>Sorts array by specified column</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="75" t="inlineStr">
+        <is>
+          <t>HSTACK</t>
+        </is>
+      </c>
+      <c r="C33" s="74" t="inlineStr">
+        <is>
+          <t>Horizontally stacks arrays into single array</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="75" t="inlineStr">
+        <is>
+          <t>LAMBDA</t>
+        </is>
+      </c>
+      <c r="C34" s="74" t="inlineStr">
+        <is>
+          <t>Creates custom reusable functions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:D2"/>

</xml_diff>